<commit_message>
implementation of formulation from chapter 3
</commit_message>
<xml_diff>
--- a/Tutorials_noted/Results/Flexures/Swan/results.xlsx
+++ b/Tutorials_noted/Results/Flexures/Swan/results.xlsx
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="7">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="97" uniqueCount="19">
   <si>
     <t>emax</t>
   </si>
@@ -38,12 +38,48 @@
   <si>
     <t>WITH ENFORCE SYMMETRY</t>
   </si>
+  <si>
+    <t>etaNormMin</t>
+  </si>
+  <si>
+    <t>etaMax</t>
+  </si>
+  <si>
+    <t>etaMaxMin</t>
+  </si>
+  <si>
+    <t>with mesh 200x200</t>
+  </si>
+  <si>
+    <t>LS</t>
+  </si>
+  <si>
+    <t>DENSITY</t>
+  </si>
+  <si>
+    <t>with initial density 0,1</t>
+  </si>
+  <si>
+    <t>LS with holes</t>
+  </si>
+  <si>
+    <t>nholes</t>
+  </si>
+  <si>
+    <t>total lengths</t>
+  </si>
+  <si>
+    <t>phases</t>
+  </si>
+  <si>
+    <t>phizero</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="2">
+  <fonts count="3">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -58,8 +94,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color rgb="FF9C6500"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -69,6 +112,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFC6EFCE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFEB9C"/>
       </patternFill>
     </fill>
   </fills>
@@ -81,16 +129,19 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Buena" xfId="1" builtinId="26"/>
+    <cellStyle name="Neutral" xfId="2" builtinId="28"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -775,6 +826,758 @@
         <a:xfrm>
           <a:off x="3962400" y="44256960"/>
           <a:ext cx="3436620" cy="3497580"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="1">
+          <a:noFill/>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd type="none" w="med" len="med"/>
+        </a:ln>
+        <a:effectLst/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>281</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>495300</xdr:colOff>
+      <xdr:row>300</xdr:row>
+      <xdr:rowOff>22860</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId15"/>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="3962400" y="51389280"/>
+          <a:ext cx="3665220" cy="3497580"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="1">
+          <a:noFill/>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd type="none" w="med" len="med"/>
+        </a:ln>
+        <a:effectLst/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>304798</xdr:colOff>
+      <xdr:row>272</xdr:row>
+      <xdr:rowOff>125507</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>623045</xdr:colOff>
+      <xdr:row>303</xdr:row>
+      <xdr:rowOff>125319</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="7" name="Picture 2"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId16"/>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="8193739" y="48893507"/>
+          <a:ext cx="11362765" cy="5557930"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="1">
+          <a:noFill/>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd type="none" w="med" len="med"/>
+        </a:ln>
+        <a:effectLst/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>320</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>236220</xdr:colOff>
+      <xdr:row>338</xdr:row>
+      <xdr:rowOff>121920</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="8" name="Picture 3"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId17"/>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="3962400" y="58521600"/>
+          <a:ext cx="3406140" cy="3413760"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="1">
+          <a:noFill/>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd type="none" w="med" len="med"/>
+        </a:ln>
+        <a:effectLst/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>672353</xdr:colOff>
+      <xdr:row>309</xdr:row>
+      <xdr:rowOff>170330</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>665629</xdr:colOff>
+      <xdr:row>342</xdr:row>
+      <xdr:rowOff>18491</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="9" name="Picture 4"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId18"/>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="7772400" y="55572212"/>
+          <a:ext cx="11826688" cy="5764867"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="1">
+          <a:noFill/>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd type="none" w="med" len="med"/>
+        </a:ln>
+        <a:effectLst/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>363</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>9</xdr:col>
+      <xdr:colOff>335280</xdr:colOff>
+      <xdr:row>382</xdr:row>
+      <xdr:rowOff>38100</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="10" name="Picture 5"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId19"/>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="3962400" y="66385440"/>
+          <a:ext cx="3505200" cy="3512820"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="1">
+          <a:noFill/>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd type="none" w="med" len="med"/>
+        </a:ln>
+        <a:effectLst/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>17929</xdr:colOff>
+      <xdr:row>351</xdr:row>
+      <xdr:rowOff>161365</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>276560</xdr:colOff>
+      <xdr:row>384</xdr:row>
+      <xdr:rowOff>117396</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1030" name="Picture 6"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId20"/>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="7906870" y="63093600"/>
+          <a:ext cx="12092043" cy="5872737"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="1">
+          <a:noFill/>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd type="none" w="med" len="med"/>
+        </a:ln>
+        <a:effectLst/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>358588</xdr:colOff>
+      <xdr:row>396</xdr:row>
+      <xdr:rowOff>35860</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>166743</xdr:colOff>
+      <xdr:row>425</xdr:row>
+      <xdr:rowOff>20519</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1031" name="Picture 7"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId21"/>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="8247529" y="71036331"/>
+          <a:ext cx="10852673" cy="5184188"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="1">
+          <a:noFill/>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd type="none" w="med" len="med"/>
+        </a:ln>
+        <a:effectLst/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>5</xdr:col>
+      <xdr:colOff>654424</xdr:colOff>
+      <xdr:row>404</xdr:row>
+      <xdr:rowOff>80683</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>109370</xdr:colOff>
+      <xdr:row>423</xdr:row>
+      <xdr:rowOff>15689</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1032" name="Picture 8"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId22"/>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="4598895" y="72515507"/>
+          <a:ext cx="3399416" cy="3341594"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="1">
+          <a:noFill/>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd type="none" w="med" len="med"/>
+        </a:ln>
+        <a:effectLst/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>573741</xdr:colOff>
+      <xdr:row>437</xdr:row>
+      <xdr:rowOff>98612</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>25</xdr:col>
+      <xdr:colOff>350071</xdr:colOff>
+      <xdr:row>468</xdr:row>
+      <xdr:rowOff>148743</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1033" name="Picture 9"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId23"/>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="8462682" y="78450141"/>
+          <a:ext cx="11609742" cy="5608249"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="1">
+          <a:noFill/>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd type="none" w="med" len="med"/>
+        </a:ln>
+        <a:effectLst/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>448</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>182880</xdr:colOff>
+      <xdr:row>466</xdr:row>
+      <xdr:rowOff>60960</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="1034" name="Picture 10"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId24"/>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="4754880" y="81930240"/>
+          <a:ext cx="3352800" cy="3352800"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="1">
+          <a:noFill/>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd type="none" w="med" len="med"/>
+        </a:ln>
+        <a:effectLst/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>489</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>300920</xdr:colOff>
+      <xdr:row>508</xdr:row>
+      <xdr:rowOff>8964</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="11" name="Picture 1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId25"/>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="4733365" y="87674824"/>
+          <a:ext cx="3456496" cy="3415552"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="1">
+          <a:noFill/>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd type="none" w="med" len="med"/>
+        </a:ln>
+        <a:effectLst/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>690282</xdr:colOff>
+      <xdr:row>478</xdr:row>
+      <xdr:rowOff>89647</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>24</xdr:col>
+      <xdr:colOff>107128</xdr:colOff>
+      <xdr:row>510</xdr:row>
+      <xdr:rowOff>24653</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="12" name="Picture 2"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId26"/>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="8579223" y="85792235"/>
+          <a:ext cx="10461364" cy="5672418"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="1">
+          <a:noFill/>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd type="none" w="med" len="med"/>
+        </a:ln>
+        <a:effectLst/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>779930</xdr:colOff>
+      <xdr:row>517</xdr:row>
+      <xdr:rowOff>2</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>786203</xdr:colOff>
+      <xdr:row>550</xdr:row>
+      <xdr:rowOff>135967</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="13" name="Picture 1"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId27"/>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="8668871" y="92695061"/>
+          <a:ext cx="12628579" cy="6052671"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="1">
+          <a:noFill/>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd type="none" w="med" len="med"/>
+        </a:ln>
+        <a:effectLst/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>530</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>213360</xdr:colOff>
+      <xdr:row>548</xdr:row>
+      <xdr:rowOff>99060</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="14" name="Picture 2"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId28"/>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="4754880" y="96926400"/>
+          <a:ext cx="3383280" cy="3390900"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="1">
+          <a:noFill/>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd type="none" w="med" len="med"/>
+        </a:ln>
+        <a:effectLst/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>699247</xdr:colOff>
+      <xdr:row>559</xdr:row>
+      <xdr:rowOff>98611</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>26</xdr:col>
+      <xdr:colOff>481404</xdr:colOff>
+      <xdr:row>592</xdr:row>
+      <xdr:rowOff>63796</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="15" name="Picture 3"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId29"/>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="8588188" y="100324023"/>
+          <a:ext cx="12404463" cy="5881891"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+        <a:noFill/>
+        <a:ln w="1">
+          <a:noFill/>
+          <a:miter lim="800000"/>
+          <a:headEnd/>
+          <a:tailEnd type="none" w="med" len="med"/>
+        </a:ln>
+        <a:effectLst/>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>6</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>569</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>10</xdr:col>
+      <xdr:colOff>320040</xdr:colOff>
+      <xdr:row>588</xdr:row>
+      <xdr:rowOff>30480</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="16" name="Picture 4"/>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId30"/>
+        <a:srcRect/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr bwMode="auto">
+        <a:xfrm>
+          <a:off x="4754880" y="104058720"/>
+          <a:ext cx="3489960" cy="3505200"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -1079,7 +1882,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="F5:T279"/>
+  <dimension ref="F5:X610"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4"/>
   <sheetData>
     <row r="5" spans="6:7">
@@ -1424,6 +2227,460 @@
       </c>
       <c r="I279">
         <v>500</v>
+      </c>
+    </row>
+    <row r="313" spans="6:7">
+      <c r="F313" t="s">
+        <v>0</v>
+      </c>
+      <c r="G313">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="314" spans="6:7">
+      <c r="F314" t="s">
+        <v>3</v>
+      </c>
+      <c r="G314">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="315" spans="6:7">
+      <c r="F315" t="s">
+        <v>7</v>
+      </c>
+      <c r="G315">
+        <v>5.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="316" spans="6:7">
+      <c r="F316" t="s">
+        <v>2</v>
+      </c>
+      <c r="G316">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="317" spans="6:7">
+      <c r="F317" t="s">
+        <v>8</v>
+      </c>
+      <c r="G317">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="318" spans="6:7">
+      <c r="F318" t="s">
+        <v>9</v>
+      </c>
+      <c r="G318">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="356" spans="7:8">
+      <c r="G356" t="s">
+        <v>0</v>
+      </c>
+      <c r="H356">
+        <v>5.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="357" spans="7:8">
+      <c r="G357" t="s">
+        <v>3</v>
+      </c>
+      <c r="H357">
+        <v>0.02</v>
+      </c>
+    </row>
+    <row r="358" spans="7:8">
+      <c r="G358" t="s">
+        <v>7</v>
+      </c>
+      <c r="H358">
+        <v>5.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="359" spans="7:8">
+      <c r="G359" t="s">
+        <v>2</v>
+      </c>
+      <c r="H359">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="360" spans="7:8">
+      <c r="G360" t="s">
+        <v>8</v>
+      </c>
+      <c r="H360">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="361" spans="7:8">
+      <c r="G361" t="s">
+        <v>9</v>
+      </c>
+      <c r="H361">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="397" spans="7:8">
+      <c r="G397" t="s">
+        <v>0</v>
+      </c>
+      <c r="H397">
+        <v>5.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="398" spans="7:8">
+      <c r="G398" t="s">
+        <v>3</v>
+      </c>
+      <c r="H398">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="399" spans="7:8">
+      <c r="G399" t="s">
+        <v>7</v>
+      </c>
+      <c r="H399">
+        <v>1E-3</v>
+      </c>
+    </row>
+    <row r="400" spans="7:8">
+      <c r="G400" t="s">
+        <v>2</v>
+      </c>
+      <c r="H400">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="401" spans="7:8">
+      <c r="G401" t="s">
+        <v>8</v>
+      </c>
+      <c r="H401">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="402" spans="7:8">
+      <c r="G402" t="s">
+        <v>9</v>
+      </c>
+      <c r="H402">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="440" spans="7:8">
+      <c r="G440" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="441" spans="7:8">
+      <c r="G441" t="s">
+        <v>0</v>
+      </c>
+      <c r="H441">
+        <v>7.4999999999999997E-3</v>
+      </c>
+    </row>
+    <row r="442" spans="7:8">
+      <c r="G442" t="s">
+        <v>1</v>
+      </c>
+      <c r="H442">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="443" spans="7:8">
+      <c r="G443" t="s">
+        <v>3</v>
+      </c>
+      <c r="H443">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="444" spans="7:8">
+      <c r="G444" t="s">
+        <v>2</v>
+      </c>
+      <c r="H444">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="445" spans="7:8">
+      <c r="G445" t="s">
+        <v>5</v>
+      </c>
+      <c r="H445">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="481" spans="7:8">
+      <c r="G481" t="s">
+        <v>0</v>
+      </c>
+      <c r="H481">
+        <v>5.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="482" spans="7:8">
+      <c r="G482" t="s">
+        <v>3</v>
+      </c>
+      <c r="H482">
+        <v>7.4999999999999997E-3</v>
+      </c>
+    </row>
+    <row r="483" spans="7:8">
+      <c r="G483" t="s">
+        <v>7</v>
+      </c>
+      <c r="H483">
+        <v>1E-4</v>
+      </c>
+    </row>
+    <row r="484" spans="7:8">
+      <c r="G484" t="s">
+        <v>2</v>
+      </c>
+      <c r="H484">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="485" spans="7:8">
+      <c r="G485" t="s">
+        <v>8</v>
+      </c>
+      <c r="H485">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="486" spans="7:8">
+      <c r="G486" t="s">
+        <v>9</v>
+      </c>
+      <c r="H486">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="515" spans="7:24">
+      <c r="G515" s="2"/>
+      <c r="H515" s="2"/>
+      <c r="I515" s="2"/>
+      <c r="J515" s="2"/>
+      <c r="K515" s="2"/>
+      <c r="L515" s="2"/>
+      <c r="M515" s="2"/>
+      <c r="N515" s="2"/>
+      <c r="O515" s="2"/>
+      <c r="P515" s="2"/>
+      <c r="Q515" s="2"/>
+      <c r="R515" s="2"/>
+      <c r="S515" s="2"/>
+      <c r="T515" s="2"/>
+      <c r="U515" s="2"/>
+      <c r="V515" s="2"/>
+      <c r="W515" s="2"/>
+      <c r="X515" s="2"/>
+    </row>
+    <row r="520" spans="7:24">
+      <c r="G520" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="521" spans="7:24">
+      <c r="G521" t="s">
+        <v>0</v>
+      </c>
+      <c r="H521">
+        <v>5.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="522" spans="7:24">
+      <c r="G522" t="s">
+        <v>3</v>
+      </c>
+      <c r="H522">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="523" spans="7:24">
+      <c r="G523" t="s">
+        <v>7</v>
+      </c>
+      <c r="H523">
+        <v>5.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="524" spans="7:24">
+      <c r="G524" t="s">
+        <v>2</v>
+      </c>
+      <c r="H524">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="525" spans="7:24">
+      <c r="G525" t="s">
+        <v>8</v>
+      </c>
+      <c r="H525">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="526" spans="7:24">
+      <c r="G526" t="s">
+        <v>9</v>
+      </c>
+      <c r="H526">
+        <v>0.01</v>
+      </c>
+    </row>
+    <row r="561" spans="7:8">
+      <c r="G561" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="562" spans="7:8">
+      <c r="G562" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="563" spans="7:8">
+      <c r="G563" t="s">
+        <v>0</v>
+      </c>
+      <c r="H563">
+        <v>7.4999999999999997E-3</v>
+      </c>
+    </row>
+    <row r="564" spans="7:8">
+      <c r="G564" t="s">
+        <v>1</v>
+      </c>
+      <c r="H564">
+        <v>500</v>
+      </c>
+    </row>
+    <row r="565" spans="7:8">
+      <c r="G565" t="s">
+        <v>3</v>
+      </c>
+      <c r="H565">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="566" spans="7:8">
+      <c r="G566" t="s">
+        <v>2</v>
+      </c>
+      <c r="H566">
+        <v>0.05</v>
+      </c>
+    </row>
+    <row r="567" spans="7:8">
+      <c r="G567" t="s">
+        <v>5</v>
+      </c>
+      <c r="H567">
+        <v>300</v>
+      </c>
+    </row>
+    <row r="599" spans="7:9">
+      <c r="G599" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="600" spans="7:9">
+      <c r="G600" t="s">
+        <v>15</v>
+      </c>
+      <c r="H600">
+        <v>80</v>
+      </c>
+      <c r="I600">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="601" spans="7:9">
+      <c r="G601" t="s">
+        <v>16</v>
+      </c>
+      <c r="H601">
+        <v>1</v>
+      </c>
+      <c r="I601">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="602" spans="7:9">
+      <c r="G602" t="s">
+        <v>17</v>
+      </c>
+      <c r="H602">
+        <v>0</v>
+      </c>
+      <c r="I602">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="603" spans="7:9">
+      <c r="G603" t="s">
+        <v>18</v>
+      </c>
+      <c r="H603">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="605" spans="7:9">
+      <c r="G605" t="s">
+        <v>0</v>
+      </c>
+      <c r="H605">
+        <v>5.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="606" spans="7:9">
+      <c r="G606" t="s">
+        <v>3</v>
+      </c>
+      <c r="H606">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="607" spans="7:9">
+      <c r="G607" t="s">
+        <v>7</v>
+      </c>
+      <c r="H607">
+        <v>5.0000000000000001E-3</v>
+      </c>
+    </row>
+    <row r="608" spans="7:9">
+      <c r="G608" t="s">
+        <v>2</v>
+      </c>
+      <c r="H608">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="609" spans="7:8">
+      <c r="G609" t="s">
+        <v>8</v>
+      </c>
+      <c r="H609">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="610" spans="7:8">
+      <c r="G610" t="s">
+        <v>9</v>
+      </c>
+      <c r="H610">
+        <v>0.01</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added norm for input-output prescribed motion
Now the norm of the vector [input output] prescribed displacements is always 1 so that cases with different values of J are comparable.
</commit_message>
<xml_diff>
--- a/Tutorials_noted/Results/Flexures/Swan/results.xlsx
+++ b/Tutorials_noted/Results/Flexures/Swan/results.xlsx
@@ -2539,6 +2539,24 @@
         <v>0.01</v>
       </c>
     </row>
+    <row r="555" spans="7:13">
+      <c r="G555" s="2"/>
+      <c r="H555" s="2"/>
+      <c r="I555" s="2"/>
+      <c r="J555" s="2"/>
+      <c r="K555" s="2"/>
+      <c r="L555" s="2"/>
+      <c r="M555" s="2"/>
+    </row>
+    <row r="556" spans="7:13">
+      <c r="G556" s="2"/>
+      <c r="H556" s="2"/>
+      <c r="I556" s="2"/>
+      <c r="J556" s="2"/>
+      <c r="K556" s="2"/>
+      <c r="L556" s="2"/>
+      <c r="M556" s="2"/>
+    </row>
     <row r="561" spans="7:8">
       <c r="G561" t="s">
         <v>12</v>

</xml_diff>